<commit_message>
Atualizacao automatica (14/03/2026  7:40:04,64)
</commit_message>
<xml_diff>
--- a/rejeito.xlsx
+++ b/rejeito.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PLANILHAS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A6DFE4AE-9797-4347-9E50-26601CF1040B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{10E71E57-8314-4230-9CB1-CDC84E649159}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3240" yWindow="3240" windowWidth="21600" windowHeight="11295" xr2:uid="{91E89078-AA4C-474D-B912-6FF611353892}"/>
+    <workbookView xWindow="3930" yWindow="3930" windowWidth="21600" windowHeight="11295" xr2:uid="{089D0EF2-2B28-4237-98C7-43B0F519A118}"/>
   </bookViews>
   <sheets>
     <sheet name="rejeito" sheetId="1" r:id="rId1"/>
@@ -972,7 +972,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3AA45F3-C7AE-4783-97EB-8C6A289F7541}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A3F16FD-8BD2-4DD8-9334-60B5DB251526}">
   <dimension ref="A1:O142"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>

</xml_diff>